<commit_message>
Golden Path FG: full re-run on v109.24 (both paths, numbers unchanged), green 'changed this round' flags
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-golden-path-fg-countertop-custom.xlsx
+++ b/client-docs/test-cases/emg-o-golden-path-fg-countertop-custom.xlsx
@@ -664,7 +664,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>บรรทัดสินค้า จำนวน 1.00 หน่วย ตร.ม. ราคา 12,000.00 · ยอดก่อน VAT 12,000.00 VAT 7% 840.00 · ท้ายบรรทัดมีไอคอนรายชิ้นงาน (ตัวอย่างจริง S00215)</t>
+          <t>บรรทัดสินค้า จำนวน 1.00 หน่วย ตร.ม. ราคา 12,000.00 · ยอดก่อน VAT 12,000.00 VAT 7% 840.00 · ท้ายบรรทัดมีไอคอนรายชิ้นงาน (ตัวอย่างจริง S00626)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>ขอบของชิ้นงานเรียก A, B, C, D มองจากด้านบน: A = ด้านกว้างบน, B = ด้านยาวขวา, C = ด้านกว้างล่าง, D = ด้านยาวซ้าย · ระบบคำนวณความยาวขอบให้เอง เลือกด้านไหนความยาวก็ตามด้านนั้น (ตอนรันรอบ 2 ผู้ทดสอบเลือกด้านต่างไป ได้ขอบ 3.05 ม. ยอดรวม 48,714.43 บาท ส่วนอื่นเหมือนกัน)</t>
+          <t>ขอบของชิ้นงานเรียก A, B, C, D มองจากด้านบน: A = ด้านกว้างบน, B = ด้านยาวขวา, C = ด้านกว้างล่าง, D = ด้านยาวซ้าย · ระบบคำนวณความยาวขอบให้เอง เลือกด้านไหนความยาวก็ตามด้านนั้น (ตอนรันรอบ 2 ของ 11 ต.ค. ผู้ทดสอบเลือกด้านต่างไป ได้ขอบ 3.05 ม. ยอดรวม 48,714.43 บาท ส่วนอื่นเหมือนกัน)</t>
         </is>
       </c>
       <c r="I6" s="7" t="n"/>
@@ -813,7 +813,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>ใบสั่งผลิตสถานะ Draft ชื่อแนว EG01/STFG/xxxxx (ตัวอย่างจริง EG01/STFG/00060) ป้าย "ผลิต FG จาก Slab" ผูกกับบรรทัดใบขาย · การ์ดแสดง "ต้องใช้ 3.83 ตร.ม." และ "Slab ที่เลือก 7.50 ตร.ม." ป้ายเขียว "พอ" · แถบเหลืองบอกให้กด "ย้ายไปสถานีตัด" ก่อน Confirm · แท็บผลผลิต FG มี 3 แถว (2.40 × 0.65, 1.20 × 0.60, 2.00 × 0.60) พร้อมหมายเหตุงานขอบและงานเจาะให้ช่างอ่าน</t>
+          <t>ใบสั่งผลิตสถานะ Draft ชื่อแนว EG01/STFG/xxxxx (ตัวอย่างจริง EG01/STFG/00156) ป้าย "ผลิต FG จาก Slab" ผูกกับบรรทัดใบขาย · การ์ดแสดง "ต้องใช้ 3.83 ตร.ม." และ "Slab ที่เลือก 7.50 ตร.ม." ป้ายเขียว "พอ" · แถบเหลืองบอกให้กด "ย้ายไปสถานีตัด" ก่อน Confirm · แท็บผลผลิต FG มี 3 แถว (2.40 × 0.65, 1.20 × 0.60, 2.00 × 0.60) พร้อมหมายเหตุงานขอบและงานเจาะให้ช่างอ่าน</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Slab ที่ระบบเลือก = BLK-26-0006-24 และ -25 (แผ่นละ 3.00 × 1.25 ม. รวม 7.50 ตร.ม.)</t>
+          <t>Slab ที่ระบบเลือก = BLK-26-0006-34 และ -35 (แผ่นละ 3.00 × 1.25 ม. รวม 7.50 ตร.ม.)</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -867,7 +867,8 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>ตั้งแต่ 11 ต.ค. 2569 แท็บ Components แสดงเฉพาะ Slab ที่ระบบเลือกจริง (Polished, 2 cm) — ก่อนแก้ จะมีแถว "Honed, 3 cm" ป้ายแดง Not Available ค้างอยู่ ซึ่งลูกค้าเห็นแล้วเข้าใจผิดว่าของไม่พอ</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — รันซ้ำแล้ว: แถว Components แสดงเฉพาะ Slab ที่เลือกจริง ป้ายเขียว Available (การแก้เมื่อ 11 ต.ค. ถูก commit และ deploy แล้ว)
+ตั้งแต่ 11 ต.ค. 2569 แท็บ Components แสดงเฉพาะ Slab ที่ระบบเลือกจริง (Polished, 2 cm) — ก่อนแก้ จะมีแถว "Honed, 3 cm" ป้ายแดง Not Available ค้างอยู่ ซึ่งลูกค้าเห็นแล้วเข้าใจผิดว่าของไม่พอ</t>
         </is>
       </c>
       <c r="I8" s="7" t="n"/>
@@ -905,7 +906,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>ข้อความ "Complete FG Production สำเร็จ ... ผลิตสำเร็จ 3.48 หน่วย" · สถานะ Done · ได้ FG 3 Lot (ตัวอย่าง FG-EG01/STFG/00061-01 = 2.40 × 0.65 · -02 = 1.20 × 0.60 · -03 = 2.00 × 0.60) อยู่ที่ EG01/Stock/Stone FG รวม 3.48 ตร.ม. · มูลค่าวัสดุ FG 2,430.00 บาท (Slab 2 แผ่น) · มีสมาร์ทปุ่ม Traceability / Product Moves</t>
+          <t>ข้อความ "Complete FG Production สำเร็จ ... ผลิตสำเร็จ 3.48 หน่วย" · สถานะ Done · ได้ FG 3 Lot (ตัวอย่าง FG-EG01/STFG/00156-01 = 2.40 × 0.65 · -02 = 1.20 × 0.60 · -03 = 2.00 × 0.60) อยู่ที่ EG01/Stock/Stone FG รวม 3.48 ตร.ม. · มูลค่าวัสดุ FG 2,430.00 บาท (Slab 2 แผ่น) · มีสมาร์ทปุ่ม Traceability / Product Moves</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -953,7 +954,7 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Details แสดง 3 แถวจาก Stone FG: -01 (1.56), -02 (0.72), -03 (1.20) รวม 3.48 ตร.ม. ไม่มี Lot ของงานอื่น · ใบส่งของเป็น Done Demand 3.48 Quantity 3.48 ตร.ม. และใบขายคอลัมน์ Delivered เป็น 3.48 (ตัวอย่างจริง EG01/OUT/00110)</t>
+          <t>Details แสดง 3 แถวจาก Stone FG: -01 (1.56), -02 (0.72), -03 (1.20) รวม 3.48 ตร.ม. ไม่มี Lot ของงานอื่น · ใบส่งของเป็น Done Demand 3.48 Quantity 3.48 ตร.ม. และใบขายคอลัมน์ Delivered เป็น 3.48 (ตัวอย่างจริง EG01/OUT/00333)</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -963,7 +964,8 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>⚠ ก่อนแก้ (11 ต.ค. 2569) ใบส่งของ Countertop อาจจอง FG ของงานเก่าปน แล้วขึ้นป้ายแดง Not Available ต้องลบแถวผิดและเพิ่ม Lot ที่ถูกเอง · หลังแก้ ระบบจองเฉพาะ Lot ที่ใบสั่งผลิตของบรรทัดนี้ผลิตให้ครบเอง แต่ยังควรเปิด Details ดูก่อน Validate ทุกครั้ง · ต้องส่งของ (Done) ก่อนจึงออกใบแจ้งหนี้ได้ ถ้ากด Create Invoice ก่อน ระบบแจ้ง "No items are available to invoice"</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — รันซ้ำแล้ว: ใบส่งของจองเฉพาะ Lot ของใบสั่งผลิตนี้ (3 แถว) ไม่มี Lot งานอื่นปน (การแก้เมื่อ 11 ต.ค. ถูก commit และ deploy แล้ว)
+⚠ ก่อนแก้ (11 ต.ค. 2569) ใบส่งของ Countertop อาจจอง FG ของงานเก่าปน แล้วขึ้นป้ายแดง Not Available ต้องลบแถวผิดและเพิ่ม Lot ที่ถูกเอง · หลังแก้ ระบบจองเฉพาะ Lot ที่ใบสั่งผลิตของบรรทัดนี้ผลิตให้ครบเอง แต่ยังควรเปิด Details ดูก่อน Validate ทุกครั้ง · ต้องส่งของ (Done) ก่อนจึงออกใบแจ้งหนี้ได้ ถ้ากด Create Invoice ก่อน ระบบแจ้ง "No items are available to invoice"</t>
         </is>
       </c>
       <c r="I10" s="7" t="n"/>
@@ -1001,7 +1003,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้ Posted ยอดก่อน VAT 45,720.00, VAT 3,200.40, รวม 48,920.40 · เครดิต 411100 รายได้ 4 บรรทัด (41,760 / 1,260 / 1,500 / 1,200) · เครดิต 213200 ภาษีขาย 3,200.40 · เดบิต 112100 ลูกหนี้ 48,920.40 · เดบิต 511110 ต้นทุนขาย 2,430.00 เครดิต 113150 สินค้าคงเหลือ Stone FG 2,430.00 (ตรงกับต้นทุน FG) (ตัวอย่างจริง INV/2026/00025)</t>
+          <t>ใบแจ้งหนี้ Posted ยอดก่อน VAT 45,720.00, VAT 3,200.40, รวม 48,920.40 · เครดิต 411100 รายได้ 4 บรรทัด (41,760 / 1,260 / 1,500 / 1,200) · เครดิต 213200 ภาษีขาย 3,200.40 · เดบิต 112100 ลูกหนี้ 48,920.40 · เดบิต 511110 ต้นทุนขาย 2,430.00 เครดิต 113150 สินค้าคงเหลือ Stone FG 2,430.00 (ตรงกับต้นทุน FG) (ตัวอย่างจริง INV/2026/00032)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1009,7 +1011,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H11" s="7" t="n"/>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — ปริมาณบนบรรทัดใบแจ้งหนี้แสดง 3 ตำแหน่ง (เช่น 3.480 ตร.ม., 3.600 ม.) เพราะรอบ Block ตั้งทศนิยมบรรทัดบิลเป็น 3 ตำแหน่งทั้งระบบ ยอดเงินไม่เปลี่ยน
+</t>
+        </is>
+      </c>
       <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="n"/>
       <c r="K11" s="7" t="n"/>
@@ -1197,7 +1204,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ยอดก่อน VAT 150,000.00, VAT 7% 10,500.00, รวม 160,500.00 · บรรทัดสินค้ามีไอคอน "โหลด BOQ" และ "ดูสูตร" · ต้นทุน/ชิ้น (ประมาณ) ยังเป็น 0.00 เพราะยังไม่ได้โหลดสูตร (ตัวอย่างจริง S00217)</t>
+          <t>ยอดก่อน VAT 150,000.00, VAT 7% 10,500.00, รวม 160,500.00 · บรรทัดสินค้ามีไอคอน "โหลด BOQ" และ "ดูสูตร" · ต้นทุน/ชิ้น (ประมาณ) ยังเป็น 0.00 เพราะยังไม่ได้โหลดสูตร (ตัวอย่างจริง S00627)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1293,7 +1300,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>ได้ใบสั่งผลิต 3 ใบ สถานะ Draft: งานประกอบ EG01/STFG/00062 (3.00 Units, ป้าย "งานกำหนดเอง (Custom)") · ใบตัดหิน NERO EG01/STCPL/00020 (12 ชิ้น = 4 × 3) · ใบตัดหิน GP EG01/STCPL/00021 (18 ชิ้น = 6 × 3) · Components ของงานประกอบมี กาว/epoxy 2.70 ตร.ม. และ ซีลแลนท์ 2.70 ตร.ม. ป้ายเขียว Available</t>
+          <t>ได้ใบสั่งผลิต 3 ใบ สถานะ Draft: งานประกอบ EG01/STFG/00157 (3.00 Units, ป้าย "งานกำหนดเอง (Custom)") · ใบตัดหิน NERO EG01/STCPL/00115 (12 ชิ้น = 4 × 3) · ใบตัดหิน GP EG01/STCPL/00116 (18 ชิ้น = 6 × 3) · Components ของงานประกอบมี กาว/epoxy 2.70 ตร.ม. และ ซีลแลนท์ 2.70 ตร.ม. ป้ายเขียว Available</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1429,7 +1436,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>1. ที่ใบงานประกอบ กดสมาร์ทปุ่ม "แผนตัด" เปิด EG01/STCPL/00020 (NERO)
+          <t>1. ที่ใบงานประกอบ กดสมาร์ทปุ่ม "แผนตัด" เปิด EG01/STCPL/00115 (NERO)
 2. ตรวจแท็บ "Slab ที่จะตัด" กดปุ่ม "ย้ายไปสถานีตัด" แล้ว Confirm
 3. เปิดแท็บ "ชิ้นงาน (แผน/จริง)" กดปุ่ม "คัดลอกแผนเป็นขนาดจริง"
 4. กดปุ่ม "ถอดแบบเสร็จ"</t>
@@ -1437,13 +1444,13 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Slab ที่ระบบเลือก = BLK-26-0002-23 (2.00 × 0.90 ม.)
+          <t>Slab ที่ระบบเลือก = BLK-26-0002-25 (2.00 × 0.90 ม.)
 ชิ้นงาน 12 ชิ้น: 0.45 × 0.30 และ 0.30 × 0.15 หนา 0.02 อย่างละ 6 ชิ้น</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ข้อความ "ย้ายสำเร็จ 1 lot ไป Stone Production" · หลังกดปุ่มคัดลอก ช่อง "จริง L / จริง H / จริง ความหนา" ครบทุกแถวเท่าแผน · ใบเป็น Done การ์ด "แผน 1.08 ตร.ม. ตัดได้จริง 1.08 ตร.ม." · ได้ WIP Lot CUT-EG01/STCPL/00020 จำนวน 12 ชิ้น ที่ Stone Production มูลค่า 2,899.80 บาท · ช่อง "ป้อนให้งานประกอบ" = EG01/STFG/00062</t>
+          <t>ข้อความ "ย้ายสำเร็จ 1 lot ไป Stone Production" · หลังกดปุ่มคัดลอก ช่อง "จริง L / จริง H / จริง ความหนา" ครบทุกแถวเท่าแผน · ใบเป็น Done การ์ด "แผน 1.08 ตร.ม. ตัดได้จริง 1.08 ตร.ม." · ได้ WIP Lot CUT-EG01/STCPL/00115 จำนวน 12 ชิ้น ที่ Stone Production มูลค่า 2,899.80 บาท · ช่อง "ป้อนให้งานประกอบ" = EG01/STFG/00157</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1453,7 +1460,8 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>ปุ่ม "คัดลอกแผนเป็นขนาดจริง" (เพิ่มเมื่อ 11 ต.ค. 2569) เติมขนาดจริงจากแผนให้ทุกแถวที่ยังว่างในครั้งเดียว แล้วช่างแก้เฉพาะชิ้นที่ตัดไม่ตรงแบบ ค่าที่กรอกไว้แล้วไม่ถูกทับ · ไม่ได้บันทึกเศษที่เหลือ ต้นทุน Slab ทั้งแผ่นจึงเข้า WIP ทั้งหมด (2,899.80 สูงกว่าประมาณการสูตร 579.96 × 3 = 1,739.88)</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — รันซ้ำแล้ว: ปุ่ม "คัดลอกแผนเป็นขนาดจริง" ใช้งานได้ใน v109.24 (commit และ deploy แล้ว) ตัวเลข WIP 2,899.80 เท่าเดิม
+ปุ่ม "คัดลอกแผนเป็นขนาดจริง" (เพิ่มเมื่อ 11 ต.ค. 2569) เติมขนาดจริงจากแผนให้ทุกแถวที่ยังว่างในครั้งเดียว แล้วช่างแก้เฉพาะชิ้นที่ตัดไม่ตรงแบบ ค่าที่กรอกไว้แล้วไม่ถูกทับ · ไม่ได้บันทึกเศษที่เหลือ ต้นทุน Slab ทั้งแผ่นจึงเข้า WIP ทั้งหมด (2,899.80 สูงกว่าประมาณการสูตร 579.96 × 3 = 1,739.88)</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -1479,7 +1487,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>1. กลับที่ใบงานประกอบ กดสมาร์ทปุ่ม "แผนตัด" เปิด EG01/STCPL/00021 (GP)
+          <t>1. กลับที่ใบงานประกอบ กดสมาร์ทปุ่ม "แผนตัด" เปิด EG01/STCPL/00116 (GP)
 2. ย้ายไปสถานีตัด และ Confirm
 3. แท็บ "ชิ้นงาน (แผน/จริง)" กดปุ่ม "คัดลอกแผนเป็นขนาดจริง"
 4. กดปุ่ม "ถอดแบบเสร็จ"</t>
@@ -1487,13 +1495,13 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Slab ที่ระบบเลือก = BLK-26-0006-28
+          <t>Slab ที่ระบบเลือก = BLK-26-0006-36
 ชิ้นงาน 18 ชิ้น: 0.20 × 0.45 (12 ชิ้น) และ 0.30 × 0.30 (6 ชิ้น) หนา 0.02</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ใบเป็น Done จำนวน 18.00 · แผน 1.62 ตร.ม. · ได้ WIP Lot CUT-EG01/STCPL/00021 จำนวน 18 ชิ้น ที่ Stone Production มูลค่า 1,215.00 บาท (Slab ทั้งแผ่น)</t>
+          <t>ใบเป็น Done จำนวน 18.00 · แผน 1.62 ตร.ม. · ได้ WIP Lot CUT-EG01/STCPL/00116 จำนวน 18 ชิ้น ที่ Stone Production มูลค่า 1,215.00 บาท (Slab ทั้งแผ่น)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1503,7 +1511,8 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>ปุ่มคัดลอกเติมเฉพาะช่องที่ว่าง — ถ้าแก้แถวหนึ่งเอง ปุ่มไม่ทับค่านั้น (ทดสอบแล้ว) · ถ้าช่างพิมพ์ขนาดจริงใหญ่กว่าแผน การ์ด "ตัดได้จริง" จะสูงกว่าแผน แต่ต้นทุนไม่เปลี่ยน เพราะต้นทุนคิดจาก Slab ที่ใช้จริง</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — รันซ้ำแล้ว: WIP 1,215.00 เท่าเดิม
+ปุ่มคัดลอกเติมเฉพาะช่องที่ว่าง — ถ้าแก้แถวหนึ่งเอง ปุ่มไม่ทับค่านั้น (ทดสอบแล้ว) · ถ้าช่างพิมพ์ขนาดจริงใหญ่กว่าแผน การ์ด "ตัดได้จริง" จะสูงกว่าแผน แต่ต้นทุนไม่เปลี่ยน เพราะต้นทุนคิดจาก Slab ที่ใช้จริง</t>
         </is>
       </c>
       <c r="I5" s="7" t="n"/>
@@ -1529,7 +1538,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>1. เปิดใบงานประกอบ EG01/STFG/00062 กด Confirm
+          <t>1. เปิดใบงานประกอบ EG01/STFG/00157 กด Confirm
 2. ตรวจแท็บ Components
 3. กดปุ่ม "Produce All"</t>
         </is>
@@ -1541,7 +1550,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Component Status = Available · ช่อง "Lot จาก Cutting Plan" แสดง CUT-EG01/STCPL/00020 และ 00021 · Components: กาว/epoxy 2.70 ตร.ม., ซีลแลนท์ 2.70 ตร.ม., WIP NERO 12, WIP GP 18 · หลัง Produce All สถานะ Done Quantity 3.00 / 3.00 มีสมาร์ทปุ่ม Serial Numbers 3 · ได้ FG เจดีย์บัว 3 ชิ้น (Serial ตัวอย่าง CB-00025 ถึง -27) มูลค่าวัสดุ 4,506.30 บาท (= 2,899.80 + 1,215.00 + 324.00 + 67.50) ชิ้นละ 1,502.10</t>
+          <t>Component Status = Available · ช่อง "Lot จาก Cutting Plan" แสดง CUT-EG01/STCPL/00115 และ 00116 · Components: กาว/epoxy 2.70 ตร.ม., ซีลแลนท์ 2.70 ตร.ม., WIP NERO 12, WIP GP 18 · หลัง Produce All สถานะ Done Quantity 3.00 / 3.00 มีสมาร์ทปุ่ม Serial Numbers 3 · ได้ FG เจดีย์บัว 3 ชิ้น (Serial ตัวอย่าง CB-00031 ถึง -33) มูลค่าวัสดุ 4,506.30 บาท (= 2,899.80 + 1,215.00 + 324.00 + 67.50) ชิ้นละ 1,502.10</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1551,7 +1560,8 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Confirm งานประกอบไม่ได้จนกว่าใบตัดหินที่ผูกกันทุกใบจะ Done · ใบงานประกอบที่ Done แล้วมีปุ่ม Unbuild (ยังไม่ได้ทดลอง)</t>
+          <t>[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — รันซ้ำแล้ว: Component Status = Available หลัง Confirm งานประกอบ มูลค่า FG 4,506.30 เท่าเดิม
+Confirm งานประกอบไม่ได้จนกว่าใบตัดหินที่ผูกกันทุกใบจะ Done · ใบงานประกอบที่ Done แล้วมีปุ่ม Unbuild (ยังไม่ได้ทดลอง)</t>
         </is>
       </c>
       <c r="I6" s="7" t="n"/>
@@ -1589,7 +1599,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Details แสดง Serial 3 ตัวจาก EG01/Stock/Stone FG ตัวละ 1.00 Units (ไม่มี FG ของงานอื่นปน) · ใบส่งของ Done Demand 3.00 Quantity 3.00 Units (ตัวอย่างจริง EG01/OUT/00111) · ใบขาย Delivered = 3.00</t>
+          <t>Details แสดง Serial 3 ตัวจาก EG01/Stock/Stone FG ตัวละ 1.00 Units (ไม่มี FG ของงานอื่นปน) · ใบส่งของ Done Demand 3.00 Quantity 3.00 Units (ตัวอย่างจริง EG01/OUT/00334) · ใบขาย Delivered = 3.00</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1637,7 +1647,7 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้ Posted ยอดก่อน VAT 150,000.00, VAT 7% 10,500.00, รวม 160,500.00 · เครดิต 411100 รายได้ 150,000.00 · เครดิต 213200 ภาษีขาย 10,500.00 · เดบิต 112100 ลูกหนี้ 160,500.00 · เดบิต 511110 ต้นทุนขาย 4,506.30 เครดิต 113150 สินค้าคงเหลือ Stone FG 4,506.30 (ต้นทุนวัสดุของ FG ไม่รวมค่าแรง) (ตัวอย่างจริง INV/2026/00027)</t>
+          <t>ใบแจ้งหนี้ Posted ยอดก่อน VAT 150,000.00, VAT 7% 10,500.00, รวม 160,500.00 · เครดิต 411100 รายได้ 150,000.00 · เครดิต 213200 ภาษีขาย 10,500.00 · เดบิต 112100 ลูกหนี้ 160,500.00 · เดบิต 511110 ต้นทุนขาย 4,506.30 เครดิต 113150 สินค้าคงเหลือ Stone FG 4,506.30 (ต้นทุนวัสดุของ FG ไม่รวมค่าแรง) (ตัวอย่างจริง INV/2026/00033)</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -1645,7 +1655,12 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H8" s="7" t="n"/>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[แก้/เพิ่ม] รอบ 14 ต.ค. 2569 (v109.24) — ปริมาณบนบรรทัดใบแจ้งหนี้แสดง 3 ตำแหน่ง ยอดเงินไม่เปลี่ยน
+</t>
+        </is>
+      </c>
       <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="n"/>
       <c r="K8" s="7" t="n"/>
@@ -1670,7 +1685,7 @@
       <c r="D9" s="7" t="inlineStr">
         <is>
           <t>1. เปิดแอป Accounting &gt; Accounting &gt; Journal Entries
-2. ค้นหา "FG Production Labor" ของงานประกอบ EG01/STFG/00062
+2. ค้นหา "FG Production Labor" ของงานประกอบ EG01/STFG/00157
 3. เปิดรายการ ดูเดบิตและเครดิต</t>
         </is>
       </c>
@@ -1681,7 +1696,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>รายการ MISC/2026/10/0026 "FG Production Labor — EG01/STFG/00062" เดบิต 511120 ค่าแรง 70,493.70 เครดิต 212300 (บัญชีค้างจ่ายค่าแรง) 70,493.70 (= 50% × 150,000 − 4,506.30) · ค่าแรงนี้ไม่รวมอยู่ในต้นทุนขาย 4,506.30 ของใบแจ้งหนี้</t>
+          <t>รายการ MISC/2026/10/0034 "FG Production Labor — EG01/STFG/00157" เดบิต 511120 ค่าแรง 70,493.70 เครดิต 212300 (บัญชีค้างจ่ายค่าแรง) 70,493.70 (= 50% × 150,000 − 4,506.30) · ค่าแรงนี้ไม่รวมอยู่ในต้นทุนขาย 4,506.30 ของใบแจ้งหนี้</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">

</xml_diff>